<commit_message>
Exceptions view with 3-layer trace, configurable rules, how-it-works guide, start-here card, UX audit
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/past-projects.xlsx
+++ b/samples/past-projects.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -442,10 +442,15 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>Actual Delivery</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Lead Time</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -469,15 +474,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>2023-04-10</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>2023-05-08</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>90 days</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Delivered</t>
         </is>
@@ -501,15 +511,20 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t>2023-09-05</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
           <t>2023-09-29</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>12 weeks</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Delivered</t>
         </is>
@@ -533,15 +548,20 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
+          <t>2023-05-15</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
           <t>2023-06-26</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>10 weeks</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Delivered</t>
         </is>
@@ -565,15 +585,20 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
+          <t>2023-10-02</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
           <t>2023-10-30</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>10 weeks</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Delivered</t>
         </is>
@@ -597,15 +622,20 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
+          <t>2023-03-01</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
           <t>2023-03-20</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>84</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Delivered</t>
         </is>
@@ -629,15 +659,20 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
+          <t>2023-06-01</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
           <t>2023-06-12</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>84</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>Delivered</t>
         </is>
@@ -666,10 +701,15 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
+          <t>2023-07-01</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
           <t>8 weeks</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>Delivered</t>
         </is>
@@ -698,10 +738,15 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
+          <t>2023-04-01</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
           <t>21</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>Delivered</t>
         </is>
@@ -725,15 +770,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
+          <t>2023-05-01</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
           <t>2023-04-28</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>14</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>Delivered</t>
         </is>
@@ -750,7 +800,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -771,10 +821,20 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>Actual Start</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Actual Finish</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Trade</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>% Complete</t>
         </is>
@@ -798,10 +858,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>2023-02-01</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2023-02-24</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>Drywall</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="G2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -823,10 +893,20 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t>2023-03-03</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2023-03-30</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>Drywall</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="G3" t="n">
         <v>1</v>
       </c>
     </row>
@@ -848,10 +928,20 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
+          <t>2023-03-06</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2023-03-17</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t>Paint</t>
         </is>
       </c>
-      <c r="E4" t="n">
+      <c r="G4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -873,10 +963,20 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
+          <t>2023-04-03</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2023-04-12</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
           <t>Paint</t>
         </is>
       </c>
-      <c r="E5" t="n">
+      <c r="G5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -898,10 +998,20 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
+          <t>2023-06-27</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2023-08-04</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t>Millwork</t>
         </is>
       </c>
-      <c r="E6" t="n">
+      <c r="G6" t="n">
         <v>1</v>
       </c>
     </row>
@@ -923,10 +1033,20 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
+          <t>2023-05-09</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2023-06-02</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
           <t>Electrical</t>
         </is>
       </c>
-      <c r="E7" t="n">
+      <c r="G7" t="n">
         <v>1</v>
       </c>
     </row>
@@ -948,10 +1068,20 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
+          <t>2023-04-05</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2023-04-14</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
           <t>Ceilings</t>
         </is>
       </c>
-      <c r="E8" t="n">
+      <c r="G8" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1102,7 +1232,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1110,7 +1240,11 @@
           <t>2023-05-02</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Held at 9 ft</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
           <t>Architect</t>

</xml_diff>